<commit_message>
Fix badge visibility in dark mode
</commit_message>
<xml_diff>
--- a/data/attendance.xlsx
+++ b/data/attendance.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -522,6 +522,35 @@
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>EMP02</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-08-11 10:50:54</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
         <is>
           <t>Present</t>
         </is>

</xml_diff>

<commit_message>
Changes password and forgot password
</commit_message>
<xml_diff>
--- a/data/attendance.xlsx
+++ b/data/attendance.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,97 +462,6 @@
       <c r="G1" s="1" t="inlineStr">
         <is>
           <t>status</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>EMP01</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-08-08</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-08-08 14:18:59</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-08-08 14:32:00</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>EMP02</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-08-10 10:50:18</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>EMP02</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-08-11 10:50:54</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Present</t>
         </is>
       </c>
     </row>

</xml_diff>